<commit_message>
feat: add manual email confirmation and auto push workflow
</commit_message>
<xml_diff>
--- a/data/departments.xlsx
+++ b/data/departments.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chiehyi\OneDrive - 大豐環保科技股份有限公司\文件\Claude\Agents-人力變化\數據資料夾\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dfrecyclecom-my.sharepoint.com/personal/chiehyi_df-recycle_com_tw/Documents/文件/Claude/Agents-人力變化/數據資料夾/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98F986A-B385-4A9F-B3B8-3DA6CB3749D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="14_{27784AB8-CE49-4701-80DC-87B654782C78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0382F771-F88D-4706-BF09-6C38765DD0DF}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{523536E6-F8D0-4B46-9468-A7DB43A681DC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{523536E6-F8D0-4B46-9468-A7DB43A681DC}"/>
   </bookViews>
   <sheets>
     <sheet name="處別" sheetId="1" r:id="rId1"/>
     <sheet name="職務" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">處別!$A$1:$B$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">處別!$A$1:$B$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">職務!$B$1:$C$76</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="203">
   <si>
     <t>部門名稱</t>
   </si>
@@ -749,6 +749,22 @@
   </si>
   <si>
     <t>再生處理部-宏偉</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>智能數位部</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI應用發展課</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>資安數位課</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>全興處理課</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -756,7 +772,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -812,6 +828,18 @@
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -917,7 +945,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -943,6 +971,8 @@
     <xf numFmtId="49" fontId="8" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -958,6 +988,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1247,7 +1281,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A19ACCB-7D22-40CC-882C-C167E6E93AF3}">
-  <dimension ref="A1:B114"/>
+  <dimension ref="A1:B118"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="23.54296875" style="2" customWidth="1"/>
@@ -1288,16 +1322,16 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
+      <c r="A5" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>2</v>
@@ -1305,55 +1339,55 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>11</v>
+      <c r="A10" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>15</v>
@@ -1361,7 +1395,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>15</v>
@@ -1369,7 +1403,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>15</v>
@@ -1377,7 +1411,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>15</v>
@@ -1385,7 +1419,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>15</v>
@@ -1393,23 +1427,23 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>15</v>
@@ -1417,15 +1451,15 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>24</v>
@@ -1433,15 +1467,15 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>2</v>
@@ -1449,31 +1483,31 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>198</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>198</v>
@@ -1481,23 +1515,23 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>198</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>7</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>7</v>
@@ -1505,7 +1539,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>7</v>
@@ -1513,7 +1547,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>7</v>
@@ -1521,15 +1555,15 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>35</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>35</v>
@@ -1537,15 +1571,15 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>13</v>
@@ -1553,7 +1587,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>13</v>
@@ -1561,39 +1595,39 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>9</v>
+        <v>199</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>9</v>
+        <v>199</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>15</v>
+        <v>199</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>15</v>
@@ -1601,7 +1635,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>15</v>
@@ -1609,15 +1643,15 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>13</v>
@@ -1625,39 +1659,39 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>13</v>
@@ -1665,7 +1699,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>13</v>
@@ -1673,7 +1707,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>13</v>
@@ -1681,7 +1715,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>13</v>
@@ -1689,7 +1723,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>13</v>
@@ -1697,31 +1731,31 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>15</v>
+        <v>199</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>11</v>
@@ -1729,7 +1763,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>11</v>
@@ -1737,7 +1771,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>11</v>
@@ -1745,55 +1779,55 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>24</v>
+        <v>199</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>13</v>
@@ -1801,7 +1835,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>13</v>
@@ -1809,7 +1843,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>13</v>
@@ -1817,7 +1851,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>13</v>
@@ -1825,55 +1859,55 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>8</v>
+        <v>199</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>73</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>73</v>
@@ -1881,23 +1915,23 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>11</v>
@@ -1905,159 +1939,159 @@
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>73</v>
+        <v>11</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>15</v>
+        <v>73</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>83</v>
+        <v>13</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>11</v>
+        <v>83</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A89" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B89" s="3" t="s">
+      <c r="A89" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="B89" s="10" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>88</v>
+        <v>24</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A100" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A101" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A100" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A101" s="4" t="s">
-        <v>97</v>
       </c>
       <c r="B101" s="3" t="s">
         <v>15</v>
@@ -2065,7 +2099,7 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B102" s="3" t="s">
         <v>15</v>
@@ -2073,7 +2107,7 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B103" s="3" t="s">
         <v>15</v>
@@ -2097,7 +2131,7 @@
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>15</v>
@@ -2105,7 +2139,7 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>15</v>
@@ -2113,63 +2147,95 @@
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>101</v>
+        <v>15</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109" s="4" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>101</v>
+        <v>15</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B110" s="3" t="s">
+      <c r="B112" s="3" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A111" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B111" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A112" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="B112" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A113" s="4" t="s">
-        <v>196</v>
+        <v>104</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A114" s="8" t="s">
-        <v>197</v>
+      <c r="A114" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="B114" s="4" t="s">
         <v>11</v>
       </c>
     </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A116" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B111" xr:uid="{00000000-0009-0000-0000-00000F000000}"/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <autoFilter ref="A1:B118" xr:uid="{00000000-0009-0000-0000-00000F000000}"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>